<commit_message>
fix: Update ignored fields in model definitions for improved clarity and accuracy
</commit_message>
<xml_diff>
--- a/printcenter/layout/Layout_PrintCenter_NFCOM_COMPLETO_TODOS_REGISTROS.xlsx
+++ b/printcenter/layout/Layout_PrintCenter_NFCOM_COMPLETO_TODOS_REGISTROS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Layout Print Center NFCOM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Layout Print Center NFCOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -66,7 +66,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -80,11 +80,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -101,6 +129,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,6 +546,10 @@
           <t>REG 00 - Header</t>
         </is>
       </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -540,7 +574,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 00</t>
+          <t>Tipo de Registro = 00</t>
         </is>
       </c>
     </row>
@@ -567,7 +601,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Nº Seq arquivo</t>
+          <t>Número Sequencial de arquivo</t>
         </is>
       </c>
     </row>
@@ -594,7 +628,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Nome Empresa</t>
+          <t>Nome da Empresa “Claro”</t>
         </is>
       </c>
     </row>
@@ -621,7 +655,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Data Geração (AAAAMMDD)</t>
+          <t>Data da Geração do Arquivo (AAAAMMDD)</t>
         </is>
       </c>
     </row>
@@ -648,7 +682,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Sigla Empresa</t>
+          <t>Sigla da Empresa</t>
         </is>
       </c>
     </row>
@@ -675,7 +709,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Endereço Empresa</t>
+          <t>Endereço da Empresa</t>
         </is>
       </c>
     </row>
@@ -702,7 +736,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Nº endereço</t>
+          <t>Número do endereço da Empresa</t>
         </is>
       </c>
     </row>
@@ -729,7 +763,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Complemento</t>
+          <t>Complemento do endereço da Empresa</t>
         </is>
       </c>
     </row>
@@ -756,7 +790,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>CEP Empresa</t>
         </is>
       </c>
     </row>
@@ -783,7 +817,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Cidade</t>
+          <t>Cidade Empresa</t>
         </is>
       </c>
     </row>
@@ -810,7 +844,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Bairro</t>
+          <t>Bairro Empresa</t>
         </is>
       </c>
     </row>
@@ -837,7 +871,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ da Empresa</t>
         </is>
       </c>
     </row>
@@ -864,7 +898,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>Inscrição Estadual Empresa</t>
         </is>
       </c>
     </row>
@@ -891,7 +925,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>Sigla da UF Empresa</t>
         </is>
       </c>
     </row>
@@ -918,7 +952,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão Social da Empresa</t>
         </is>
       </c>
     </row>
@@ -949,12 +983,17 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>REG 01 - Cliente</t>
         </is>
       </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -979,7 +1018,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 01</t>
+          <t>Tipo de Registro = 01</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1045,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Cód Cliente</t>
+          <t>Código de Cliente</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1072,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Nº CPS/Fatura</t>
+          <t>Número da CPS/Fatura (CPS + DV)</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1099,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Dt Emissão</t>
+          <t>Data da Emissão (DDMMAAAA)</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1126,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Dt Vencto</t>
+          <t>Data de Vencimento (DDMMAAAA)</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1153,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão Social do Cliente</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1180,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Endereço</t>
+          <t>Endereço do Cliente</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1207,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Município</t>
+          <t>Nome do Município</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1234,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>UF do Cliente</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1261,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>Cep do Cliente</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1288,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Bairro</t>
+          <t>Bairro do Cliente</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1315,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Tipo: 1=Fat, 2=DANFE, 3=Ambos</t>
+          <t>Indicador do tipo de cobrança : Fatura (“1”) ou DANFE (“2”)</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1342,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Mídia</t>
+          <t>Mídia;</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1369,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Tipo Doc</t>
+          <t>Tipo Documento:</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1396,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Movimento</t>
+          <t>Identifica o Movimento do Cliente</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1423,7 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Cód Centro Cobr</t>
+          <t>Cod-Centro-Cobrança</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1450,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Flag Débito Aut</t>
+          <t>Flag-Débito-Aut</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1477,7 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Nº 0800</t>
+          <t>Número  0800  Editado</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1504,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Flag Cad Entrega</t>
+          <t>Flag-Cad-Entrega ‘S’  Significa que o endereço de entrega está preenchido</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1531,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Nome Entrega</t>
+          <t>Nome-Cliente-Entrega</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1558,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>End Entrega</t>
+          <t>Endereço-Cliente-Entrega</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1585,7 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Mun Entrega</t>
+          <t>Nome-Município-Cliente-Entrega</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1612,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>UF Entrega</t>
+          <t>Uf-Cliente-Entrega</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1639,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>CEP Entrega</t>
+          <t>Cep-Cliente-Entrega</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1666,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Bairro Entrega</t>
+          <t>Bairro-Cliente-Entrega</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1693,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ-Cliente</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1720,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Ano-Mês Ref</t>
+          <t>Ano-Mês-Referência</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1747,7 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Dependência</t>
+          <t>Dependência-Cliente</t>
         </is>
       </c>
     </row>
@@ -1735,16 +1774,21 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Lote/FLAG</t>
-        </is>
-      </c>
-    </row>
+          <t>Lote da Net: Contrato –NET</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
     <row r="53" ht="25" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>REG 02 - Resumo Serviços</t>
         </is>
       </c>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -1769,7 +1813,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 02</t>
+          <t>Tipo de Registro = 02</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1840,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Sigla Serviço</t>
+          <t>Sigla do Serviço</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1867,7 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Descrição Serviço</t>
+          <t>Descrição do Serviço</t>
         </is>
       </c>
     </row>
@@ -1848,10 +1892,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E57" s="4">
+        <f> C, Quando  o  valor for negativo,</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -1877,7 +1920,7 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Valor Serviço</t>
+          <t>Valor do Serviço</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1974,7 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Vlr sem Desc Subst</t>
+          <t>Valor do Serviço sem Desconto Subst.Tribut.</t>
         </is>
       </c>
     </row>
@@ -1958,7 +2001,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Vlr Imposto</t>
+          <t>Valor do Imposto</t>
         </is>
       </c>
     </row>
@@ -1985,7 +2028,7 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>Tipo Imposto</t>
+          <t>Tipo de Imposto</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2055,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Vlr PIS</t>
+          <t>Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2082,7 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Vlr COFINS</t>
+          <t>Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2109,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Vlr FUST</t>
+          <t>Valor do FUST</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2136,7 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Vlr FUNTEL</t>
+          <t>Valor do FUNTEL</t>
         </is>
       </c>
     </row>
@@ -2124,12 +2167,17 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
     <row r="69" ht="25" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t>REG 03 - Itens Faturamento</t>
         </is>
       </c>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -2154,7 +2202,7 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 03</t>
+          <t>Tipo de Registro = 03</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2229,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Seq Item</t>
+          <t>Sequencial do Item</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2256,7 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Sigla</t>
+          <t>Sigla do Serviço</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2283,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Desc Serviço</t>
+          <t>Descrição de Serviço</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2337,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Desc Item</t>
+          <t>Descrição do item</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2364,7 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Dt Início</t>
+          <t>Data início Prestação de Serviço (DDMMAA)</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2391,7 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>Dt Fim</t>
+          <t>Data fim  Prestação de Serviço (DDMMAA)</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2418,7 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>Term Destino</t>
+          <t>Terminal Destino</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2445,7 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Local Orig</t>
+          <t>Local Origem</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2472,7 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>Local Dest</t>
+          <t>Local Destino</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2499,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Hr Início</t>
+          <t>Hora início Prestação de Serviço</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2526,7 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Hr Fim</t>
+          <t>Hora fim Prestação de Serviço</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2553,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Tipo Imposto</t>
+          <t>Tipo de Imposto</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2580,7 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Sigla País</t>
+          <t>Sigla de País</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2607,7 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Qtd Medida</t>
+          <t>Quantidade  Medida</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2634,7 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Desc Unid</t>
+          <t>Descrição da Unidade Medida</t>
         </is>
       </c>
     </row>
@@ -2611,10 +2659,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E87" s="4">
+        <f> C, quando o valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -2640,7 +2687,7 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Vlr Item</t>
+          <t>Valor do Item</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2714,7 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Cód Item</t>
+          <t>Código-Item (Cod-Tarifa-A)</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2741,7 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>Vlr Líq trunc</t>
+          <t>Valor-Líquido-Item truncado</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2768,7 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>Tipo Item</t>
+          <t>Tipo-Item</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2795,7 @@
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>Déb/Créd</t>
+          <t>INDIC-Débito-Crédito</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2822,7 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>Qtd Ligações</t>
+          <t>Quantidade de Ligações</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2849,7 @@
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>Cód Plano</t>
+          <t>Código do Plano Comercial</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2876,7 @@
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>PAS Local</t>
+          <t>PAS (Plano Alternativo de Serviço) Local</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2957,7 @@
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>Desc Plano</t>
+          <t>Descrição do Plano Comercial</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2984,7 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>Designação</t>
+          <t>Designação Original</t>
         </is>
       </c>
     </row>
@@ -2964,7 +3011,7 @@
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>Msg ANATEL</t>
+          <t>Mensagens importantes ANATEL</t>
         </is>
       </c>
     </row>
@@ -2991,7 +3038,7 @@
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>Vlr Líq s/trunc</t>
+          <t>Valor líquido item sem truncar</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3065,7 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>Dt Fim Perman</t>
+          <t>Data Término Prazo de Permanência</t>
         </is>
       </c>
     </row>
@@ -3049,12 +3096,17 @@
         </is>
       </c>
     </row>
+    <row r="104"/>
     <row r="105" ht="25" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t>REG 04 - Boleto</t>
         </is>
       </c>
+      <c r="B105" s="6" t="n"/>
+      <c r="C105" s="6" t="n"/>
+      <c r="D105" s="6" t="n"/>
+      <c r="E105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -3079,7 +3131,7 @@
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 04</t>
+          <t>Tipo de Registro = 04</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3158,7 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>Nome Banco</t>
+          <t>Nome do Banco</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3185,7 @@
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>Cód Banco</t>
+          <t>Código do Banco</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3212,7 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>Agência Cedente</t>
+          <t>Agência Cod-Cedente,</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3239,7 @@
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>Dt Documento</t>
+          <t>Data do Documento (DDMMAAAA)</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3266,7 @@
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>Nº Documento</t>
+          <t>Número do Documento</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3293,7 @@
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>Cód Espécie</t>
+          <t>Cód-Espécie Documento</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3320,7 @@
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
-          <t>Cód Aceite</t>
+          <t>Cód-Aceite</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3347,7 @@
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>Dt Processo</t>
+          <t>Data de Processamento (DDMMAAAA)</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3374,7 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>Cód Uso Banco</t>
+          <t>Cód.Uso do Banco</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3401,7 @@
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>Cód Carteira</t>
+          <t>Cód-Carteira</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3428,7 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>Nosso Nº</t>
+          <t>Cód-Nosso-Número</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3455,7 @@
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>Dt Vencto</t>
+          <t>Data de Vencimento (DDMMAAAA)</t>
         </is>
       </c>
     </row>
@@ -3428,10 +3480,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E119" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E119" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="120">
@@ -3457,7 +3508,7 @@
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>Vlr Documento</t>
+          <t>Valor do Documento</t>
         </is>
       </c>
     </row>
@@ -3482,10 +3533,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E121" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E121" s="4">
+        <f> C, Quando o valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="122">
@@ -3511,7 +3561,7 @@
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>Vlr Desconto</t>
+          <t>Valor de Desconto</t>
         </is>
       </c>
     </row>
@@ -3536,10 +3586,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E123" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E123" s="4">
+        <f> C, Quando  o   valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="124">
@@ -3565,7 +3614,7 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>Outras Deduções</t>
+          <t>Outras Deduções/Abatimentos</t>
         </is>
       </c>
     </row>
@@ -3590,10 +3639,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E125" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E125" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="126">
@@ -3619,7 +3667,7 @@
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>Mora/Multa</t>
+          <t>Mora/Multa/Juros</t>
         </is>
       </c>
     </row>
@@ -3644,10 +3692,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E127" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E127" s="4">
+        <f> C, Quando  o   valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="128">
@@ -3673,7 +3720,7 @@
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>Base 9,45%</t>
+          <t>Base Cálculo 9,45%</t>
         </is>
       </c>
     </row>
@@ -3698,10 +3745,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E129" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E129" s="4">
+        <f> C, Quando  o   valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="130">
@@ -3727,7 +3773,7 @@
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>Vlr Cobrado</t>
+          <t>Valor Cobrado</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3800,7 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>Msg 1</t>
+          <t>Mensagem que Consta no Bloqueto</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3827,7 @@
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>Msg 2</t>
+          <t>Mensagem que Consta no Bloqueto</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3854,7 @@
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>Msg 3</t>
+          <t>Mensagem que Consta no Bloqueto</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3881,7 @@
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>Cód Baixa</t>
+          <t>Cód. da Baixa</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3908,7 @@
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>Cód Barras</t>
+          <t>String do Código de Barras</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3935,7 @@
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>Linha Digitável</t>
+          <t>Linha Digitável (Código de Barras)</t>
         </is>
       </c>
     </row>
@@ -3914,10 +3960,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E137" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E137" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="138">
@@ -3943,7 +3988,7 @@
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>Vlr Fust</t>
+          <t>Valor Fust (Imposto)</t>
         </is>
       </c>
     </row>
@@ -3968,10 +4013,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E139" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E139" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="140">
@@ -3997,7 +4041,7 @@
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>Vlr Funtel</t>
+          <t>Valor  Funtel</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4068,7 @@
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ  do Cliente</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4095,7 @@
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>Cód Post</t>
+          <t>Código de Postagem</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4122,7 @@
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>Indica Fust</t>
+          <t>Indica-fust</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4149,7 @@
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>Ag Ced Format</t>
+          <t>Agencia cod-cedente Formatado</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4176,7 @@
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>Parc IR</t>
+          <t>Parcela retenção 9,45 IR</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4203,7 @@
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>Parc CSLL</t>
+          <t>Parcela retenção 9,45 CSLL</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4230,7 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>Parc COFINS</t>
+          <t>Parcela retenção 9,45 COFINS</t>
         </is>
       </c>
     </row>
@@ -4213,16 +4257,21 @@
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>Parc PIS</t>
-        </is>
-      </c>
-    </row>
+          <t>Parcela retenção 9,45 PIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="149"/>
     <row r="150" ht="25" customHeight="1">
       <c r="A150" s="3" t="inlineStr">
         <is>
           <t>REG 05 - Msgs Fatura (Mod22)</t>
         </is>
       </c>
+      <c r="B150" s="6" t="n"/>
+      <c r="C150" s="6" t="n"/>
+      <c r="D150" s="6" t="n"/>
+      <c r="E150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -4247,7 +4296,7 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 05</t>
+          <t>Tipo de Registro = 05</t>
         </is>
       </c>
     </row>
@@ -4274,7 +4323,7 @@
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>Mensagem CPS/Fatura</t>
+          <t>Mensagem da CPS/Fatura</t>
         </is>
       </c>
     </row>
@@ -4305,12 +4354,17 @@
         </is>
       </c>
     </row>
+    <row r="154"/>
     <row r="155" ht="25" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
           <t>REG 06 - Total Tributos</t>
         </is>
       </c>
+      <c r="B155" s="6" t="n"/>
+      <c r="C155" s="6" t="n"/>
+      <c r="D155" s="6" t="n"/>
+      <c r="E155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -4335,7 +4389,7 @@
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 06</t>
+          <t>Tipo de Registro = 06</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4416,7 @@
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>Vlr ICMS</t>
+          <t>Valor do ICMS</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4443,7 @@
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>Vlr ISS</t>
+          <t>Valor do ISS</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4470,7 @@
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>Vlr PIS</t>
+          <t>Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4497,7 @@
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>Vlr COFINS</t>
+          <t>Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -4474,12 +4528,17 @@
         </is>
       </c>
     </row>
+    <row r="162"/>
     <row r="163" ht="25" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
           <t>REG 07 - Códigos Oferta</t>
         </is>
       </c>
+      <c r="B163" s="6" t="n"/>
+      <c r="C163" s="6" t="n"/>
+      <c r="D163" s="6" t="n"/>
+      <c r="E163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -4504,7 +4563,7 @@
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 07</t>
+          <t>Tipo de Registro = 07</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4590,7 @@
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>Cód Oferta</t>
+          <t>Código Oferta</t>
         </is>
       </c>
     </row>
@@ -4558,7 +4617,7 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>Desc Oferta</t>
+          <t>Descrição Oferta</t>
         </is>
       </c>
     </row>
@@ -4589,12 +4648,17 @@
         </is>
       </c>
     </row>
+    <row r="168"/>
     <row r="169" ht="25" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
           <t>REG 08 - Perfil Consumo</t>
         </is>
       </c>
+      <c r="B169" s="6" t="n"/>
+      <c r="C169" s="6" t="n"/>
+      <c r="D169" s="6" t="n"/>
+      <c r="E169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -4619,7 +4683,7 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 08</t>
+          <t>Tipo de Registro = 08</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4710,7 @@
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>Ano Mês</t>
+          <t>Ano Mês Consumo (AAAAMM)</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4764,7 @@
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>Desc Tráfego</t>
+          <t>Descrição Tráfego Consumido</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4791,7 @@
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>Qtd Minutos</t>
+          <t>Quantidade de minutos Consumidos</t>
         </is>
       </c>
     </row>
@@ -4758,12 +4822,17 @@
         </is>
       </c>
     </row>
+    <row r="176"/>
     <row r="177" ht="25" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
           <t>REG 09 - Msgs Import (Mod22)</t>
         </is>
       </c>
+      <c r="B177" s="6" t="n"/>
+      <c r="C177" s="6" t="n"/>
+      <c r="D177" s="6" t="n"/>
+      <c r="E177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -4788,7 +4857,7 @@
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 09</t>
+          <t>Tipo de Registro = 09</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4884,7 @@
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>Cód Msg</t>
+          <t>Código da Mensagem da CPS/Fatura</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4911,7 @@
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>Mensagem</t>
+          <t>Mensagem da CPS/Fatura</t>
         </is>
       </c>
     </row>
@@ -4873,12 +4942,17 @@
         </is>
       </c>
     </row>
+    <row r="182"/>
     <row r="183" ht="25" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
           <t>REG 10 - Cadastro NF ICMS (Mod22)</t>
         </is>
       </c>
+      <c r="B183" s="6" t="n"/>
+      <c r="C183" s="6" t="n"/>
+      <c r="D183" s="6" t="n"/>
+      <c r="E183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -4903,7 +4977,7 @@
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 10</t>
+          <t>Tipo de Registro = 10</t>
         </is>
       </c>
     </row>
@@ -4930,7 +5004,7 @@
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>Cód Cliente</t>
+          <t>Código de Cliente</t>
         </is>
       </c>
     </row>
@@ -4957,7 +5031,7 @@
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>Nº CPS</t>
+          <t>Número da CPS/Fatura</t>
         </is>
       </c>
     </row>
@@ -4984,7 +5058,7 @@
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>End Empresa</t>
+          <t>Endereço da Empresa</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5085,7 @@
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>Cep  Empresa</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5112,7 @@
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Município</t>
+          <t>Nome Município Empresa</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5139,7 @@
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ  da  Empresa</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5166,7 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>Inscrição Estadual  Empresa</t>
         </is>
       </c>
     </row>
@@ -5119,7 +5193,7 @@
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>Msg Regime</t>
+          <t>Mensagem  Empresa</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5220,7 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>Sigla  da  UF  Empresa</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5247,7 @@
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>Nº NF</t>
+          <t>Número da Nota Fiscal</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5274,7 @@
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Série</t>
+          <t>Série da Nota Fiscal</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5301,7 @@
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>Dt Emissão</t>
+          <t>Data Emissão da Nota Fiscal (DDMMAA)</t>
         </is>
       </c>
     </row>
@@ -5254,7 +5328,7 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão Social do Cliente</t>
         </is>
       </c>
     </row>
@@ -5281,7 +5355,7 @@
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>End Fiscal</t>
+          <t>Endereço Fiscal Cliente</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5382,7 @@
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Município Cli</t>
+          <t>Município Fiscal Cliente</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5409,7 @@
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>Cód Estab</t>
+          <t>Cód. Estabelecimento</t>
         </is>
       </c>
     </row>
@@ -5362,7 +5436,7 @@
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>CNPJ Cli</t>
+          <t>CNPJ do Cliente, onde:</t>
         </is>
       </c>
     </row>
@@ -5389,7 +5463,7 @@
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>IE Cli</t>
+          <t>Inscrição Estadual Cliente</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5490,7 @@
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>UF Cli</t>
+          <t>UF  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -5443,7 +5517,7 @@
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>Dependência</t>
+          <t>Nome  Dependência</t>
         </is>
       </c>
     </row>
@@ -5470,7 +5544,7 @@
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>Cód Centro</t>
+          <t>Cód-Centro-Cobrança (não será impresso)</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5598,7 @@
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>Cód Empresa</t>
+          <t>Código da Empresa – Nota Fiscal ICMS</t>
         </is>
       </c>
     </row>
@@ -5555,12 +5629,17 @@
         </is>
       </c>
     </row>
+    <row r="209"/>
     <row r="210" ht="25" customHeight="1">
       <c r="A210" s="3" t="inlineStr">
         <is>
           <t>REG 11 - Itens ICMS (Mod22)</t>
         </is>
       </c>
+      <c r="B210" s="6" t="n"/>
+      <c r="C210" s="6" t="n"/>
+      <c r="D210" s="6" t="n"/>
+      <c r="E210" s="7" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
@@ -5585,7 +5664,7 @@
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 11</t>
+          <t>Tipo de Registro = 11</t>
         </is>
       </c>
     </row>
@@ -5612,7 +5691,7 @@
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>Desc Serviço</t>
+          <t>Descrição do Serviço</t>
         </is>
       </c>
     </row>
@@ -5639,7 +5718,7 @@
       </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
-          <t>Desc Origem</t>
+          <t>Descrição Origem</t>
         </is>
       </c>
     </row>
@@ -5691,10 +5770,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E215" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E215" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="216">
@@ -5720,7 +5798,7 @@
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>Vlr Item</t>
+          <t>Valor  do  Item</t>
         </is>
       </c>
     </row>
@@ -5747,7 +5825,7 @@
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>Código nacional de Localidade (CNL)</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5852,7 @@
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>Nº Contrato</t>
+          <t>Número contrato de vendas</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5879,7 @@
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>Vlr Imposto</t>
+          <t>Valor do Imposto</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5906,7 @@
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>Vlr PIS</t>
+          <t>Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -5855,7 +5933,7 @@
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>Vlr COFINS</t>
+          <t>Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -5886,12 +5964,17 @@
         </is>
       </c>
     </row>
+    <row r="223"/>
     <row r="224" ht="25" customHeight="1">
       <c r="A224" s="3" t="inlineStr">
         <is>
           <t>REG 12 - Base Cálc (Mod22)</t>
         </is>
       </c>
+      <c r="B224" s="6" t="n"/>
+      <c r="C224" s="6" t="n"/>
+      <c r="D224" s="6" t="n"/>
+      <c r="E224" s="7" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
@@ -5916,7 +5999,7 @@
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 12</t>
+          <t>Tipo de Registro = 12</t>
         </is>
       </c>
     </row>
@@ -5941,10 +6024,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E226" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E226" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="227">
@@ -5970,7 +6052,7 @@
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total</t>
+          <t>Valor  Total</t>
         </is>
       </c>
     </row>
@@ -5995,10 +6077,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E228" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E228" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="229">
@@ -6024,7 +6105,7 @@
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>Base Cálc</t>
+          <t>Valor da Base de Cálculo</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6132,7 @@
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>Asterisco</t>
+          <t>Asterisco Alíquota,</t>
         </is>
       </c>
     </row>
@@ -6103,10 +6184,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E232" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E232" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="233">
@@ -6132,7 +6212,7 @@
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>Vlr ICMS</t>
+          <t>Valor  do  Imposto (ICMS)</t>
         </is>
       </c>
     </row>
@@ -6157,10 +6237,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E234" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E234" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="235">
@@ -6186,7 +6265,7 @@
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>Vlr Isentos</t>
+          <t>Valor  Isentos</t>
         </is>
       </c>
     </row>
@@ -6211,10 +6290,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E236" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E236" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="237">
@@ -6240,7 +6318,7 @@
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>Vlr Outros</t>
+          <t>Valor  Outros</t>
         </is>
       </c>
     </row>
@@ -6271,12 +6349,17 @@
         </is>
       </c>
     </row>
+    <row r="239"/>
     <row r="240" ht="25" customHeight="1">
       <c r="A240" s="3" t="inlineStr">
         <is>
           <t>REG 13 - Somatórios ICMS (Mod22)</t>
         </is>
       </c>
+      <c r="B240" s="6" t="n"/>
+      <c r="C240" s="6" t="n"/>
+      <c r="D240" s="6" t="n"/>
+      <c r="E240" s="7" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
@@ -6301,7 +6384,7 @@
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 13</t>
+          <t>Tipo de Registro = 13</t>
         </is>
       </c>
     </row>
@@ -6326,10 +6409,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E242" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E242" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="243">
@@ -6355,7 +6437,7 @@
       </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
-          <t>Som Vlr Total</t>
+          <t>Somatório Valor Total</t>
         </is>
       </c>
     </row>
@@ -6380,10 +6462,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E244" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E244" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="245">
@@ -6409,7 +6490,7 @@
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>Som Base</t>
+          <t>Somatório</t>
         </is>
       </c>
     </row>
@@ -6434,10 +6515,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E246" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E246" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="247">
@@ -6463,7 +6543,7 @@
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>Som Imposto</t>
+          <t>Somatório Valor de Imposto</t>
         </is>
       </c>
     </row>
@@ -6488,10 +6568,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E248" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E248" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="249">
@@ -6517,7 +6596,7 @@
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>Som Isentos</t>
+          <t>Somatório Valor Isentos</t>
         </is>
       </c>
     </row>
@@ -6542,10 +6621,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E250" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E250" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="251">
@@ -6571,7 +6649,7 @@
       </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
-          <t>Som Outros</t>
+          <t>Somatório Valor Outros</t>
         </is>
       </c>
     </row>
@@ -6598,7 +6676,7 @@
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>Msg Rodapé 1</t>
+          <t>Mensagem Rodapé (redução de base de cálculo), caso não exista será igual a branco</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6703,7 @@
       </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
-          <t>Msg Rodapé 2</t>
+          <t>Idem</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6730,7 @@
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>Msg Rodapé 3</t>
+          <t>Idem</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6757,7 @@
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t>Hash-Code</t>
+          <t>Hash-Code editado</t>
         </is>
       </c>
     </row>
@@ -6710,12 +6788,17 @@
         </is>
       </c>
     </row>
+    <row r="257"/>
     <row r="258" ht="25" customHeight="1">
       <c r="A258" s="3" t="inlineStr">
         <is>
           <t>REG 14 - Msgs NF ICMS (Mod22)</t>
         </is>
       </c>
+      <c r="B258" s="6" t="n"/>
+      <c r="C258" s="6" t="n"/>
+      <c r="D258" s="6" t="n"/>
+      <c r="E258" s="7" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
@@ -6740,7 +6823,7 @@
       </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 14</t>
+          <t>Tipo de Registro = 14</t>
         </is>
       </c>
     </row>
@@ -6767,7 +6850,7 @@
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>Mensagem NF</t>
+          <t>Mensagem da Nota Fiscal</t>
         </is>
       </c>
     </row>
@@ -6798,12 +6881,17 @@
         </is>
       </c>
     </row>
+    <row r="262"/>
     <row r="263" ht="25" customHeight="1">
       <c r="A263" s="3" t="inlineStr">
         <is>
           <t>REG 15 - Cad Oper ICMS (Mod22)</t>
         </is>
       </c>
+      <c r="B263" s="6" t="n"/>
+      <c r="C263" s="6" t="n"/>
+      <c r="D263" s="6" t="n"/>
+      <c r="E263" s="7" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
@@ -6828,7 +6916,7 @@
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 15</t>
+          <t>Tipo de Registro = 15</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6943,7 @@
       </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
-          <t>Cód Cliente</t>
+          <t>Código de Cliente</t>
         </is>
       </c>
     </row>
@@ -6882,7 +6970,7 @@
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>Nº CPS</t>
+          <t>Número da CPS/Fatura</t>
         </is>
       </c>
     </row>
@@ -6909,7 +6997,7 @@
       </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>End Embratel</t>
+          <t>Endereço da Embratel</t>
         </is>
       </c>
     </row>
@@ -6936,7 +7024,7 @@
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>Cep  Embratel</t>
         </is>
       </c>
     </row>
@@ -6963,7 +7051,7 @@
       </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
-          <t>Município</t>
+          <t>Nome Município  Embratel</t>
         </is>
       </c>
     </row>
@@ -6990,7 +7078,7 @@
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ  da  Embratel</t>
         </is>
       </c>
     </row>
@@ -7017,7 +7105,7 @@
       </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>Inscrição Estadual  Embratel</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7132,7 @@
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>Sigla  da  UF  Embratel</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7159,7 @@
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>Dt Emissão</t>
+          <t>Data Emissão da Nota Fiscal (DDMMAA)</t>
         </is>
       </c>
     </row>
@@ -7098,7 +7186,7 @@
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão Social do Cliente</t>
         </is>
       </c>
     </row>
@@ -7125,7 +7213,7 @@
       </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
-          <t>End Fiscal</t>
+          <t>Endereço Fiscal Cliente</t>
         </is>
       </c>
     </row>
@@ -7152,7 +7240,7 @@
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>Município Cli</t>
+          <t>Município Fiscal Cliente</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7267,7 @@
       </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
-          <t>Cód Estab</t>
+          <t>Cód. Estabelecimento</t>
         </is>
       </c>
     </row>
@@ -7206,7 +7294,7 @@
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>CNPJ Cli</t>
+          <t>CNPJ do Cliente, onde:</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7348,7 @@
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>UF Cli</t>
+          <t>UF  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7375,7 @@
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>Dependência</t>
+          <t>Nome  Dependência</t>
         </is>
       </c>
     </row>
@@ -7314,7 +7402,7 @@
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>Cód Centro</t>
+          <t>Cód-Centro-Cobrança</t>
         </is>
       </c>
     </row>
@@ -7345,12 +7433,17 @@
         </is>
       </c>
     </row>
+    <row r="284"/>
     <row r="285" ht="25" customHeight="1">
       <c r="A285" s="3" t="inlineStr">
         <is>
           <t>REG 16 - Dados Oper (Mod22)</t>
         </is>
       </c>
+      <c r="B285" s="6" t="n"/>
+      <c r="C285" s="6" t="n"/>
+      <c r="D285" s="6" t="n"/>
+      <c r="E285" s="7" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
@@ -7375,7 +7468,7 @@
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 16</t>
+          <t>Tipo de Registro = 16</t>
         </is>
       </c>
     </row>
@@ -7402,7 +7495,7 @@
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>Nome Oper</t>
+          <t>Nome Operadora</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7522,7 @@
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>End Oper</t>
+          <t>Endereço da Operadora</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7549,7 @@
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>Cep Operadora</t>
         </is>
       </c>
     </row>
@@ -7483,7 +7576,7 @@
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>Município</t>
+          <t>Nome Município Operadora</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7603,7 @@
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ da Operadora</t>
         </is>
       </c>
     </row>
@@ -7537,7 +7630,7 @@
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>Inscrição Estadual da Operadora</t>
         </is>
       </c>
     </row>
@@ -7564,7 +7657,7 @@
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>Msg Regime</t>
+          <t>Mensagem (Regime Especial)</t>
         </is>
       </c>
     </row>
@@ -7591,7 +7684,7 @@
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>Sigla UF da Operadora</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7711,7 @@
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>Nº NF</t>
+          <t>Número da Nota Fiscal Operadora</t>
         </is>
       </c>
     </row>
@@ -7645,7 +7738,7 @@
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>Série</t>
+          <t>Série da Nota Fiscal Operadora</t>
         </is>
       </c>
     </row>
@@ -7672,7 +7765,7 @@
       </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
-          <t>Sub-série</t>
+          <t>Sub-série da Nota Fiscal Operadora</t>
         </is>
       </c>
     </row>
@@ -7730,12 +7823,17 @@
         </is>
       </c>
     </row>
+    <row r="300"/>
     <row r="301" ht="25" customHeight="1">
       <c r="A301" s="3" t="inlineStr">
         <is>
           <t>REG 17 - Itens Oper (Mod22)</t>
         </is>
       </c>
+      <c r="B301" s="6" t="n"/>
+      <c r="C301" s="6" t="n"/>
+      <c r="D301" s="6" t="n"/>
+      <c r="E301" s="7" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
@@ -7760,7 +7858,7 @@
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 17</t>
+          <t>Tipo de Registro = 17</t>
         </is>
       </c>
     </row>
@@ -7787,7 +7885,7 @@
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Desc Serviço</t>
+          <t>Descrição do Serviço da operadora</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7912,7 @@
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Desc Origem</t>
+          <t>Descrição Origem</t>
         </is>
       </c>
     </row>
@@ -7866,10 +7964,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E306" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E306" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="307">
@@ -7895,7 +7992,7 @@
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Vlr Item</t>
+          <t>Valor  do  Item</t>
         </is>
       </c>
     </row>
@@ -7922,7 +8019,7 @@
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>Código nacional de Localidade (CNL)</t>
         </is>
       </c>
     </row>
@@ -7949,7 +8046,7 @@
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Vlr Imposto</t>
+          <t>Valor do Imposto</t>
         </is>
       </c>
     </row>
@@ -7976,7 +8073,7 @@
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>Vlr PIS</t>
+          <t>Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -8003,7 +8100,7 @@
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Vlr COFINS</t>
+          <t>Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -8034,12 +8131,17 @@
         </is>
       </c>
     </row>
+    <row r="313"/>
     <row r="314" ht="25" customHeight="1">
       <c r="A314" s="3" t="inlineStr">
         <is>
           <t>REG 18 - Base Oper (Mod22)</t>
         </is>
       </c>
+      <c r="B314" s="6" t="n"/>
+      <c r="C314" s="6" t="n"/>
+      <c r="D314" s="6" t="n"/>
+      <c r="E314" s="7" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
@@ -8064,7 +8166,7 @@
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 18</t>
+          <t>Tipo de Registro = 18</t>
         </is>
       </c>
     </row>
@@ -8089,10 +8191,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E316" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E316" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="317">
@@ -8118,7 +8219,7 @@
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total</t>
+          <t>Valor  Total</t>
         </is>
       </c>
     </row>
@@ -8143,10 +8244,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E318" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E318" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="319">
@@ -8172,7 +8272,7 @@
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>Base Cálc</t>
+          <t>Valor da Base de Cálculo</t>
         </is>
       </c>
     </row>
@@ -8199,7 +8299,7 @@
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>Asterisco</t>
+          <t>Asterisco Alíquota,</t>
         </is>
       </c>
     </row>
@@ -8251,10 +8351,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E322" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E322" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="323">
@@ -8280,7 +8379,7 @@
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>Vlr ICMS</t>
+          <t>Valor  do  Imposto (ICMS)</t>
         </is>
       </c>
     </row>
@@ -8305,10 +8404,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E324" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E324" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="325">
@@ -8334,7 +8432,7 @@
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>Vlr Isentos</t>
+          <t>Valor  Isentos</t>
         </is>
       </c>
     </row>
@@ -8359,10 +8457,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E326" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E326" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="327">
@@ -8388,7 +8485,7 @@
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>Vlr Outros</t>
+          <t>Valor  Outros</t>
         </is>
       </c>
     </row>
@@ -8419,12 +8516,17 @@
         </is>
       </c>
     </row>
+    <row r="329"/>
     <row r="330" ht="25" customHeight="1">
       <c r="A330" s="3" t="inlineStr">
         <is>
           <t>REG 19 - Som Oper (Mod22)</t>
         </is>
       </c>
+      <c r="B330" s="6" t="n"/>
+      <c r="C330" s="6" t="n"/>
+      <c r="D330" s="6" t="n"/>
+      <c r="E330" s="7" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
@@ -8449,7 +8551,7 @@
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 19</t>
+          <t>Tipo de Registro = 19</t>
         </is>
       </c>
     </row>
@@ -8474,10 +8576,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E332" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E332" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="333">
@@ -8503,7 +8604,7 @@
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>Som Vlr Total</t>
+          <t>Somatório Valor Total</t>
         </is>
       </c>
     </row>
@@ -8528,10 +8629,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E334" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E334" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="335">
@@ -8557,7 +8657,7 @@
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>Som Base</t>
+          <t>Somatório</t>
         </is>
       </c>
     </row>
@@ -8582,10 +8682,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E336" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E336" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="337">
@@ -8611,7 +8710,7 @@
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>Som Imposto</t>
+          <t>Somatório Valor de Imposto</t>
         </is>
       </c>
     </row>
@@ -8665,7 +8764,7 @@
       </c>
       <c r="E339" s="4" t="inlineStr">
         <is>
-          <t>Som Isentos</t>
+          <t>Somatório Valor Isentos</t>
         </is>
       </c>
     </row>
@@ -8690,10 +8789,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E340" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E340" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="341">
@@ -8719,7 +8817,7 @@
       </c>
       <c r="E341" s="4" t="inlineStr">
         <is>
-          <t>Som Outros</t>
+          <t>Somatório Valor Outros</t>
         </is>
       </c>
     </row>
@@ -8746,7 +8844,7 @@
       </c>
       <c r="E342" s="4" t="inlineStr">
         <is>
-          <t>Hash-Code</t>
+          <t>Hash-Code operadora</t>
         </is>
       </c>
     </row>
@@ -8777,12 +8875,17 @@
         </is>
       </c>
     </row>
+    <row r="344"/>
     <row r="345" ht="25" customHeight="1">
       <c r="A345" s="3" t="inlineStr">
         <is>
           <t>REG 20 - Cadastro NF ISS (Mod22)</t>
         </is>
       </c>
+      <c r="B345" s="6" t="n"/>
+      <c r="C345" s="6" t="n"/>
+      <c r="D345" s="6" t="n"/>
+      <c r="E345" s="7" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="4" t="inlineStr">
@@ -8807,7 +8910,7 @@
       </c>
       <c r="E346" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 20</t>
+          <t>Tipo de Registro = 20</t>
         </is>
       </c>
     </row>
@@ -8834,7 +8937,7 @@
       </c>
       <c r="E347" s="4" t="inlineStr">
         <is>
-          <t>Cód Cliente</t>
+          <t>Código  de  Cliente</t>
         </is>
       </c>
     </row>
@@ -8861,7 +8964,7 @@
       </c>
       <c r="E348" s="4" t="inlineStr">
         <is>
-          <t>Nº NF</t>
+          <t>Número da Nota Fiscal</t>
         </is>
       </c>
     </row>
@@ -8888,7 +8991,7 @@
       </c>
       <c r="E349" s="4" t="inlineStr">
         <is>
-          <t>Cód Prefeitura</t>
+          <t>Código  da  Prefeitura</t>
         </is>
       </c>
     </row>
@@ -8915,7 +9018,7 @@
       </c>
       <c r="E350" s="4" t="inlineStr">
         <is>
-          <t>Nome Prefeitura</t>
+          <t>Nome  da  Prefeitura</t>
         </is>
       </c>
     </row>
@@ -8942,7 +9045,7 @@
       </c>
       <c r="E351" s="4" t="inlineStr">
         <is>
-          <t>Validade</t>
+          <t>Validade  de  Emissão</t>
         </is>
       </c>
     </row>
@@ -8969,7 +9072,7 @@
       </c>
       <c r="E352" s="4" t="inlineStr">
         <is>
-          <t>Natureza Op</t>
+          <t>Natureza  da  Operação</t>
         </is>
       </c>
     </row>
@@ -8996,7 +9099,7 @@
       </c>
       <c r="E353" s="4" t="inlineStr">
         <is>
-          <t>Nº Fatura</t>
+          <t>Número  da  Fatura/CPS</t>
         </is>
       </c>
     </row>
@@ -9023,7 +9126,7 @@
       </c>
       <c r="E354" s="4" t="inlineStr">
         <is>
-          <t>Dt Emissão</t>
+          <t>Data-Emissão (AAAAMMDD)</t>
         </is>
       </c>
     </row>
@@ -9050,7 +9153,7 @@
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
-          <t>Mês Ref</t>
+          <t>Mês/Ref</t>
         </is>
       </c>
     </row>
@@ -9077,7 +9180,7 @@
       </c>
       <c r="E356" s="4" t="inlineStr">
         <is>
-          <t>Cód Fiscal</t>
+          <t>Código  Fiscal</t>
         </is>
       </c>
     </row>
@@ -9104,7 +9207,7 @@
       </c>
       <c r="E357" s="4" t="inlineStr">
         <is>
-          <t>End Empresa</t>
+          <t>Endereço da Empresa</t>
         </is>
       </c>
     </row>
@@ -9131,7 +9234,7 @@
       </c>
       <c r="E358" s="4" t="inlineStr">
         <is>
-          <t>UF Emp</t>
+          <t>UF  da  Empresa</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9261,7 @@
       </c>
       <c r="E359" s="4" t="inlineStr">
         <is>
-          <t>CNPJ Emp</t>
+          <t>CNPJ  da  Empresa</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9288,7 @@
       </c>
       <c r="E360" s="4" t="inlineStr">
         <is>
-          <t>IM Emp</t>
+          <t>Inscrição  Municipal  Empresa</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9315,7 @@
       </c>
       <c r="E361" s="4" t="inlineStr">
         <is>
-          <t>IE Emp</t>
+          <t>Inscrição  Estadual  Empresa</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9342,7 @@
       </c>
       <c r="E362" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão  Social  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -9266,7 +9369,7 @@
       </c>
       <c r="E363" s="4" t="inlineStr">
         <is>
-          <t>End Fiscal</t>
+          <t>Endereço  Fiscal  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9396,7 @@
       </c>
       <c r="E364" s="4" t="inlineStr">
         <is>
-          <t>Município Cli</t>
+          <t>Município  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -9320,7 +9423,7 @@
       </c>
       <c r="E365" s="4" t="inlineStr">
         <is>
-          <t>UF Cli</t>
+          <t>UF  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -9347,7 +9450,7 @@
       </c>
       <c r="E366" s="4" t="inlineStr">
         <is>
-          <t>CNPJ Cli</t>
+          <t>CNPJ  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -9374,7 +9477,7 @@
       </c>
       <c r="E367" s="4" t="inlineStr">
         <is>
-          <t>IM Cli</t>
+          <t>Inscrição  Municipal  Cliente</t>
         </is>
       </c>
     </row>
@@ -9401,7 +9504,7 @@
       </c>
       <c r="E368" s="4" t="inlineStr">
         <is>
-          <t>IE Cli</t>
+          <t>Inscrição  Estadual  Cliente</t>
         </is>
       </c>
     </row>
@@ -9428,7 +9531,7 @@
       </c>
       <c r="E369" s="4" t="inlineStr">
         <is>
-          <t>Cód Estab</t>
+          <t>Cód.  Estabelecimento</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9558,7 @@
       </c>
       <c r="E370" s="4" t="inlineStr">
         <is>
-          <t>Cód Segurança</t>
+          <t>Código  de  Segurança</t>
         </is>
       </c>
     </row>
@@ -9482,7 +9585,7 @@
       </c>
       <c r="E371" s="4" t="inlineStr">
         <is>
-          <t>Cód Emp ISS</t>
+          <t>Código Empresa ISS - Nota Fiscal ISS (Logo e papel)</t>
         </is>
       </c>
     </row>
@@ -9509,7 +9612,7 @@
       </c>
       <c r="E372" s="4" t="inlineStr">
         <is>
-          <t>Desc Título</t>
+          <t>Descrição-título-nota-ISS</t>
         </is>
       </c>
     </row>
@@ -9536,7 +9639,7 @@
       </c>
       <c r="E373" s="4" t="inlineStr">
         <is>
-          <t>Cód Emp Princ</t>
+          <t>Código da Empresa – Nota Fiscal ISS</t>
         </is>
       </c>
     </row>
@@ -9563,7 +9666,7 @@
       </c>
       <c r="E374" s="4" t="inlineStr">
         <is>
-          <t>Cód Emp Parc</t>
+          <t>Código da Empresa – Nota Fiscal ISS</t>
         </is>
       </c>
     </row>
@@ -9594,12 +9697,17 @@
         </is>
       </c>
     </row>
+    <row r="376"/>
     <row r="377" ht="25" customHeight="1">
       <c r="A377" s="3" t="inlineStr">
         <is>
           <t>REG 21 - Itens ISS (Mod22)</t>
         </is>
       </c>
+      <c r="B377" s="6" t="n"/>
+      <c r="C377" s="6" t="n"/>
+      <c r="D377" s="6" t="n"/>
+      <c r="E377" s="7" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="4" t="inlineStr">
@@ -9624,7 +9732,7 @@
       </c>
       <c r="E378" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 21</t>
+          <t>Tipo de Registro = 21</t>
         </is>
       </c>
     </row>
@@ -9651,7 +9759,7 @@
       </c>
       <c r="E379" s="4" t="inlineStr">
         <is>
-          <t>Cód Sigla</t>
+          <t>Cód-Sigla-Serviço</t>
         </is>
       </c>
     </row>
@@ -9705,7 +9813,7 @@
       </c>
       <c r="E381" s="4" t="inlineStr">
         <is>
-          <t>Desc Item</t>
+          <t>Descrição  do Item</t>
         </is>
       </c>
     </row>
@@ -9757,10 +9865,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E383" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E383" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="384">
@@ -9786,7 +9893,7 @@
       </c>
       <c r="E384" s="4" t="inlineStr">
         <is>
-          <t>Vlr Unit</t>
+          <t>Valor  Unitário</t>
         </is>
       </c>
     </row>
@@ -9838,10 +9945,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E386" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E386" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="387">
@@ -9867,7 +9973,7 @@
       </c>
       <c r="E387" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total</t>
+          <t>Valor  Total</t>
         </is>
       </c>
     </row>
@@ -9892,10 +9998,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E388" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E388" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="389">
@@ -9921,7 +10026,7 @@
       </c>
       <c r="E389" s="4" t="inlineStr">
         <is>
-          <t>Vlr ISS</t>
+          <t>Valor  de  ISS</t>
         </is>
       </c>
     </row>
@@ -9948,7 +10053,7 @@
       </c>
       <c r="E390" s="4" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>Código nacional de Localidade (CNL)</t>
         </is>
       </c>
     </row>
@@ -9975,7 +10080,7 @@
       </c>
       <c r="E391" s="4" t="inlineStr">
         <is>
-          <t>Vlr PIS</t>
+          <t>Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -10002,7 +10107,7 @@
       </c>
       <c r="E392" s="4" t="inlineStr">
         <is>
-          <t>Vlr COFINS</t>
+          <t>Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -10033,12 +10138,17 @@
         </is>
       </c>
     </row>
+    <row r="394"/>
     <row r="395" ht="25" customHeight="1">
       <c r="A395" s="3" t="inlineStr">
         <is>
           <t>REG 22 - Total ISS (Mod22)</t>
         </is>
       </c>
+      <c r="B395" s="6" t="n"/>
+      <c r="C395" s="6" t="n"/>
+      <c r="D395" s="6" t="n"/>
+      <c r="E395" s="7" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="4" t="inlineStr">
@@ -10063,7 +10173,7 @@
       </c>
       <c r="E396" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 22</t>
+          <t>Tipo de Registro = 22</t>
         </is>
       </c>
     </row>
@@ -10088,10 +10198,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E397" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E397" s="4">
+        <f> C, Quando  o  valor for negativo</f>
+        <v/>
       </c>
     </row>
     <row r="398">
@@ -10117,7 +10226,7 @@
       </c>
       <c r="E398" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total NF</t>
+          <t>Valor  Total  da  Nota</t>
         </is>
       </c>
     </row>
@@ -10144,7 +10253,7 @@
       </c>
       <c r="E399" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total ISS</t>
+          <t>Valor-Total-ISS-Nota</t>
         </is>
       </c>
     </row>
@@ -10175,12 +10284,17 @@
         </is>
       </c>
     </row>
+    <row r="401"/>
     <row r="402" ht="25" customHeight="1">
       <c r="A402" s="3" t="inlineStr">
         <is>
           <t>REG 23 - Msgs ISS (Mod22)</t>
         </is>
       </c>
+      <c r="B402" s="6" t="n"/>
+      <c r="C402" s="6" t="n"/>
+      <c r="D402" s="6" t="n"/>
+      <c r="E402" s="7" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="4" t="inlineStr">
@@ -10205,7 +10319,7 @@
       </c>
       <c r="E403" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 23</t>
+          <t>Tipo de Registro = 23</t>
         </is>
       </c>
     </row>
@@ -10232,7 +10346,7 @@
       </c>
       <c r="E404" s="4" t="inlineStr">
         <is>
-          <t>Msg 1</t>
+          <t>Mensagem  1</t>
         </is>
       </c>
     </row>
@@ -10259,7 +10373,7 @@
       </c>
       <c r="E405" s="4" t="inlineStr">
         <is>
-          <t>Msg 2</t>
+          <t>Mensagem  2</t>
         </is>
       </c>
     </row>
@@ -10286,7 +10400,7 @@
       </c>
       <c r="E406" s="4" t="inlineStr">
         <is>
-          <t>Msg 3</t>
+          <t>Mensagem  3</t>
         </is>
       </c>
     </row>
@@ -10313,7 +10427,7 @@
       </c>
       <c r="E407" s="4" t="inlineStr">
         <is>
-          <t>Msg 4</t>
+          <t>Mensagem  4</t>
         </is>
       </c>
     </row>
@@ -10340,7 +10454,7 @@
       </c>
       <c r="E408" s="4" t="inlineStr">
         <is>
-          <t>Msg 5</t>
+          <t>Mensagem  5</t>
         </is>
       </c>
     </row>
@@ -10367,7 +10481,7 @@
       </c>
       <c r="E409" s="4" t="inlineStr">
         <is>
-          <t>Msg 6</t>
+          <t>Mensagem  6</t>
         </is>
       </c>
     </row>
@@ -10398,12 +10512,17 @@
         </is>
       </c>
     </row>
+    <row r="411"/>
     <row r="412" ht="25" customHeight="1">
       <c r="A412" s="3" t="inlineStr">
         <is>
           <t>REG 24 - Rodapé ISS (Mod22)</t>
         </is>
       </c>
+      <c r="B412" s="6" t="n"/>
+      <c r="C412" s="6" t="n"/>
+      <c r="D412" s="6" t="n"/>
+      <c r="E412" s="7" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="4" t="inlineStr">
@@ -10428,7 +10547,7 @@
       </c>
       <c r="E413" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 24</t>
+          <t>Tipo de Registro = 24</t>
         </is>
       </c>
     </row>
@@ -10455,7 +10574,7 @@
       </c>
       <c r="E414" s="4" t="inlineStr">
         <is>
-          <t>Cód AIDF</t>
+          <t>Código  AIDF</t>
         </is>
       </c>
     </row>
@@ -10486,12 +10605,17 @@
         </is>
       </c>
     </row>
+    <row r="416"/>
     <row r="417" ht="25" customHeight="1">
       <c r="A417" s="3" t="inlineStr">
         <is>
           <t>REG 30 - Recibo (Mod22)</t>
         </is>
       </c>
+      <c r="B417" s="6" t="n"/>
+      <c r="C417" s="6" t="n"/>
+      <c r="D417" s="6" t="n"/>
+      <c r="E417" s="7" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="4" t="inlineStr">
@@ -10516,7 +10640,7 @@
       </c>
       <c r="E418" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 30</t>
+          <t>Tipo de Registro = 30</t>
         </is>
       </c>
     </row>
@@ -10543,7 +10667,7 @@
       </c>
       <c r="E419" s="4" t="inlineStr">
         <is>
-          <t>Cód Cliente</t>
+          <t>Código  do  Cliente</t>
         </is>
       </c>
     </row>
@@ -10570,7 +10694,7 @@
       </c>
       <c r="E420" s="4" t="inlineStr">
         <is>
-          <t>Nº Recibo</t>
+          <t>Número  do  Recibo (AAMMLLLXXXXX)</t>
         </is>
       </c>
     </row>
@@ -10597,7 +10721,7 @@
       </c>
       <c r="E421" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão  Social</t>
         </is>
       </c>
     </row>
@@ -10624,7 +10748,7 @@
       </c>
       <c r="E422" s="4" t="inlineStr">
         <is>
-          <t>End Cobrança</t>
+          <t>Endereço  Cobrança</t>
         </is>
       </c>
     </row>
@@ -10651,7 +10775,7 @@
       </c>
       <c r="E423" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>UF-Cobrança</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10856,7 @@
       </c>
       <c r="E426" s="4" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>Inscrição  Estadual</t>
         </is>
       </c>
     </row>
@@ -10759,7 +10883,7 @@
       </c>
       <c r="E427" s="4" t="inlineStr">
         <is>
-          <t>IM</t>
+          <t>Inscrição  Municipal</t>
         </is>
       </c>
     </row>
@@ -10786,7 +10910,7 @@
       </c>
       <c r="E428" s="4" t="inlineStr">
         <is>
-          <t>Nº CPS</t>
+          <t>Número  CPS</t>
         </is>
       </c>
     </row>
@@ -10813,7 +10937,7 @@
       </c>
       <c r="E429" s="4" t="inlineStr">
         <is>
-          <t>Dt Emissão</t>
+          <t>Data  Emissão (DDMMAAAA)</t>
         </is>
       </c>
     </row>
@@ -10844,12 +10968,17 @@
         </is>
       </c>
     </row>
+    <row r="431"/>
     <row r="432" ht="25" customHeight="1">
       <c r="A432" s="3" t="inlineStr">
         <is>
           <t>REG 31 - Itens Recibo (Mod22)</t>
         </is>
       </c>
+      <c r="B432" s="6" t="n"/>
+      <c r="C432" s="6" t="n"/>
+      <c r="D432" s="6" t="n"/>
+      <c r="E432" s="7" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="4" t="inlineStr">
@@ -10874,7 +11003,7 @@
       </c>
       <c r="E433" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 31</t>
+          <t>Tipo de Registro = 31</t>
         </is>
       </c>
     </row>
@@ -10901,7 +11030,7 @@
       </c>
       <c r="E434" s="4" t="inlineStr">
         <is>
-          <t>Sigla Serv</t>
+          <t>Sigla  de  Serviço</t>
         </is>
       </c>
     </row>
@@ -10928,7 +11057,7 @@
       </c>
       <c r="E435" s="4" t="inlineStr">
         <is>
-          <t>Desc Serv</t>
+          <t>Descrição  Serviço</t>
         </is>
       </c>
     </row>
@@ -10953,10 +11082,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E436" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E436" s="4">
+        <f> C, Quando  o  valor for negativo,</f>
+        <v/>
       </c>
     </row>
     <row r="437">
@@ -11013,12 +11141,17 @@
         </is>
       </c>
     </row>
+    <row r="439"/>
     <row r="440" ht="25" customHeight="1">
       <c r="A440" s="3" t="inlineStr">
         <is>
           <t>REG 32 - Som Recibo (Mod22)</t>
         </is>
       </c>
+      <c r="B440" s="6" t="n"/>
+      <c r="C440" s="6" t="n"/>
+      <c r="D440" s="6" t="n"/>
+      <c r="E440" s="7" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="4" t="inlineStr">
@@ -11043,7 +11176,7 @@
       </c>
       <c r="E441" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 32</t>
+          <t>Tipo de Registro = 32</t>
         </is>
       </c>
     </row>
@@ -11068,10 +11201,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E442" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E442" s="4">
+        <f> C, Quando  o  valor for negativo,</f>
+        <v/>
       </c>
     </row>
     <row r="443">
@@ -11097,7 +11229,7 @@
       </c>
       <c r="E443" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total</t>
+          <t>Valor-Total</t>
         </is>
       </c>
     </row>
@@ -11128,12 +11260,17 @@
         </is>
       </c>
     </row>
+    <row r="445"/>
     <row r="446" ht="25" customHeight="1">
       <c r="A446" s="3" t="inlineStr">
         <is>
           <t>REG 40 - Cadastro NFCOM</t>
         </is>
       </c>
+      <c r="B446" s="6" t="n"/>
+      <c r="C446" s="6" t="n"/>
+      <c r="D446" s="6" t="n"/>
+      <c r="E446" s="7" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="4" t="inlineStr">
@@ -11158,7 +11295,7 @@
       </c>
       <c r="E447" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 40</t>
+          <t>Tipo de Registro = 40</t>
         </is>
       </c>
     </row>
@@ -11185,7 +11322,7 @@
       </c>
       <c r="E448" s="4" t="inlineStr">
         <is>
-          <t>Cód Cliente</t>
+          <t>Código de Cliente</t>
         </is>
       </c>
     </row>
@@ -11212,7 +11349,7 @@
       </c>
       <c r="E449" s="4" t="inlineStr">
         <is>
-          <t>Nº CPS</t>
+          <t>Número da CPS/Fatura</t>
         </is>
       </c>
     </row>
@@ -11239,7 +11376,7 @@
       </c>
       <c r="E450" s="4" t="inlineStr">
         <is>
-          <t>End Empresa</t>
+          <t>Endereço da Empresa</t>
         </is>
       </c>
     </row>
@@ -11266,7 +11403,7 @@
       </c>
       <c r="E451" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>Cep  Empresa</t>
         </is>
       </c>
     </row>
@@ -11293,7 +11430,7 @@
       </c>
       <c r="E452" s="4" t="inlineStr">
         <is>
-          <t>Município</t>
+          <t>Nome Município Empresa</t>
         </is>
       </c>
     </row>
@@ -11320,7 +11457,7 @@
       </c>
       <c r="E453" s="4" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>CNPJ  da  Empresa</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11484,7 @@
       </c>
       <c r="E454" s="4" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>Inscrição Estadual  Empresa</t>
         </is>
       </c>
     </row>
@@ -11374,7 +11511,7 @@
       </c>
       <c r="E455" s="4" t="inlineStr">
         <is>
-          <t>Msg Regime</t>
+          <t>Mensagem  Empresa (Regime Especial)</t>
         </is>
       </c>
     </row>
@@ -11401,7 +11538,7 @@
       </c>
       <c r="E456" s="4" t="inlineStr">
         <is>
-          <t>UF</t>
+          <t>Sigla  da  UF  Empresa</t>
         </is>
       </c>
     </row>
@@ -11428,7 +11565,7 @@
       </c>
       <c r="E457" s="4" t="inlineStr">
         <is>
-          <t>Nº NF</t>
+          <t>Número da Nota Fiscal</t>
         </is>
       </c>
     </row>
@@ -11455,7 +11592,7 @@
       </c>
       <c r="E458" s="4" t="inlineStr">
         <is>
-          <t>Série</t>
+          <t>Série da Nota Fiscal</t>
         </is>
       </c>
     </row>
@@ -11482,7 +11619,7 @@
       </c>
       <c r="E459" s="4" t="inlineStr">
         <is>
-          <t>Dt Emissão</t>
+          <t>Data Emissão da Nota Fiscal (DDMMAA)</t>
         </is>
       </c>
     </row>
@@ -11509,7 +11646,7 @@
       </c>
       <c r="E460" s="4" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Razão Social do Cliente</t>
         </is>
       </c>
     </row>
@@ -11536,7 +11673,7 @@
       </c>
       <c r="E461" s="4" t="inlineStr">
         <is>
-          <t>End Fiscal</t>
+          <t>Endereço Fiscal Cliente</t>
         </is>
       </c>
     </row>
@@ -11563,7 +11700,7 @@
       </c>
       <c r="E462" s="4" t="inlineStr">
         <is>
-          <t>Município Cli</t>
+          <t>Município Fiscal Cliente</t>
         </is>
       </c>
     </row>
@@ -11590,7 +11727,7 @@
       </c>
       <c r="E463" s="4" t="inlineStr">
         <is>
-          <t>Cód Estab</t>
+          <t>Cód. Estabelecimento</t>
         </is>
       </c>
     </row>
@@ -11617,7 +11754,7 @@
       </c>
       <c r="E464" s="4" t="inlineStr">
         <is>
-          <t>CNPJ/CPF</t>
+          <t>CNPJ do Cliente / CPF do Cliente</t>
         </is>
       </c>
     </row>
@@ -11644,7 +11781,7 @@
       </c>
       <c r="E465" s="4" t="inlineStr">
         <is>
-          <t>IE Cli</t>
+          <t>Inscrição Estadual Cliente</t>
         </is>
       </c>
     </row>
@@ -11671,7 +11808,7 @@
       </c>
       <c r="E466" s="4" t="inlineStr">
         <is>
-          <t>UF Cli</t>
+          <t>UF do Cliente</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11835,7 @@
       </c>
       <c r="E467" s="4" t="inlineStr">
         <is>
-          <t>Dependência</t>
+          <t>Nome Dependência</t>
         </is>
       </c>
     </row>
@@ -11725,7 +11862,7 @@
       </c>
       <c r="E468" s="4" t="inlineStr">
         <is>
-          <t>Cód Centro</t>
+          <t>Cód-Centro-Cobrança (não será impresso)</t>
         </is>
       </c>
     </row>
@@ -11779,7 +11916,7 @@
       </c>
       <c r="E470" s="4" t="inlineStr">
         <is>
-          <t>Cód Empresa</t>
+          <t>Código da Empresa – Nota Fiscal ICMS  (Logo principal)= EBT (EMBRATEL), = NSC (STARONE), = CLO (CLARO), = TLM (TELMEX)</t>
         </is>
       </c>
     </row>
@@ -11806,16 +11943,21 @@
       </c>
       <c r="E471" s="4" t="inlineStr">
         <is>
-          <t>Gerar Ficha (S/N)</t>
-        </is>
-      </c>
-    </row>
+          <t>(S)im/(N)ão === Gerar Ficha Arrecadação</t>
+        </is>
+      </c>
+    </row>
+    <row r="472"/>
     <row r="473" ht="25" customHeight="1">
       <c r="A473" s="3" t="inlineStr">
         <is>
           <t>REG 42 - Compl 40 (1/2)</t>
         </is>
       </c>
+      <c r="B473" s="6" t="n"/>
+      <c r="C473" s="6" t="n"/>
+      <c r="D473" s="6" t="n"/>
+      <c r="E473" s="7" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="4" t="inlineStr">
@@ -11840,7 +11982,7 @@
       </c>
       <c r="E474" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 42</t>
+          <t>Tipo de Registro = 42</t>
         </is>
       </c>
     </row>
@@ -11867,7 +12009,7 @@
       </c>
       <c r="E475" s="4" t="inlineStr">
         <is>
-          <t>Telefone</t>
+          <t>Telefone Principal</t>
         </is>
       </c>
     </row>
@@ -11894,7 +12036,7 @@
       </c>
       <c r="E476" s="4" t="inlineStr">
         <is>
-          <t>Bairro</t>
+          <t>Bairro Cliente</t>
         </is>
       </c>
     </row>
@@ -11921,7 +12063,7 @@
       </c>
       <c r="E477" s="4" t="inlineStr">
         <is>
-          <t>CEP</t>
+          <t>Cep Cliente</t>
         </is>
       </c>
     </row>
@@ -11948,7 +12090,7 @@
       </c>
       <c r="E478" s="4" t="inlineStr">
         <is>
-          <t>Dt Início Ciclo</t>
+          <t>Data INICIAL do ciclo de consumo do cliente da fatura (Competência).</t>
         </is>
       </c>
     </row>
@@ -11975,7 +12117,7 @@
       </c>
       <c r="E479" s="4" t="inlineStr">
         <is>
-          <t>Dt Fim Ciclo</t>
+          <t>Data FINAL do ciclo de consumo do cliente da fatura (Competência).</t>
         </is>
       </c>
     </row>
@@ -12056,7 +12198,7 @@
       </c>
       <c r="E482" s="4" t="inlineStr">
         <is>
-          <t>Total Pagar</t>
+          <t>Total a Pagar (Valor Cobrado)</t>
         </is>
       </c>
     </row>
@@ -12137,7 +12279,7 @@
       </c>
       <c r="E485" s="4" t="inlineStr">
         <is>
-          <t>Link Consulta</t>
+          <t>Link para Consulta pela Chave de Acesso</t>
         </is>
       </c>
     </row>
@@ -12164,7 +12306,7 @@
       </c>
       <c r="E486" s="4" t="inlineStr">
         <is>
-          <t>Chave Acesso</t>
+          <t>Chave de acesso da NFCom emitida pela operadora local.</t>
         </is>
       </c>
     </row>
@@ -12191,7 +12333,7 @@
       </c>
       <c r="E487" s="4" t="inlineStr">
         <is>
-          <t>Nº Protocolo</t>
+          <t>Número do protocolo de autorização do documento NFCOM</t>
         </is>
       </c>
     </row>
@@ -12218,7 +12360,7 @@
       </c>
       <c r="E488" s="4" t="inlineStr">
         <is>
-          <t>Dt Protocolo</t>
+          <t>Data do Protocolo de Autorização</t>
         </is>
       </c>
     </row>
@@ -12245,7 +12387,7 @@
       </c>
       <c r="E489" s="4" t="inlineStr">
         <is>
-          <t>Hr Protocolo</t>
+          <t>Hora do Protocolo de Autorização</t>
         </is>
       </c>
     </row>
@@ -12276,12 +12418,17 @@
         </is>
       </c>
     </row>
+    <row r="491"/>
     <row r="492" ht="25" customHeight="1">
       <c r="A492" s="3" t="inlineStr">
         <is>
           <t>REG 44 - Compl 40 (2/2)</t>
         </is>
       </c>
+      <c r="B492" s="6" t="n"/>
+      <c r="C492" s="6" t="n"/>
+      <c r="D492" s="6" t="n"/>
+      <c r="E492" s="7" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="4" t="inlineStr">
@@ -12306,7 +12453,7 @@
       </c>
       <c r="E493" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 44</t>
+          <t>Tipo de Registro = 44</t>
         </is>
       </c>
     </row>
@@ -12333,7 +12480,7 @@
       </c>
       <c r="E494" s="4" t="inlineStr">
         <is>
-          <t>URL QRCode NF (até 1000b, 4 regs max)</t>
+          <t>URL do QRCode apresentado na fatura.</t>
         </is>
       </c>
     </row>
@@ -12364,12 +12511,17 @@
         </is>
       </c>
     </row>
+    <row r="496"/>
     <row r="497" ht="25" customHeight="1">
       <c r="A497" s="3" t="inlineStr">
         <is>
           <t>REG 46 - Itens NFCOM</t>
         </is>
       </c>
+      <c r="B497" s="6" t="n"/>
+      <c r="C497" s="6" t="n"/>
+      <c r="D497" s="6" t="n"/>
+      <c r="E497" s="7" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="4" t="inlineStr">
@@ -12394,7 +12546,7 @@
       </c>
       <c r="E498" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 46</t>
+          <t>Tipo de Registro = 46</t>
         </is>
       </c>
     </row>
@@ -12421,7 +12573,7 @@
       </c>
       <c r="E499" s="4" t="inlineStr">
         <is>
-          <t>Desc Serviço</t>
+          <t>Descrição do Serviço</t>
         </is>
       </c>
     </row>
@@ -12448,7 +12600,7 @@
       </c>
       <c r="E500" s="4" t="inlineStr">
         <is>
-          <t>Desc Origem</t>
+          <t>Descrição Origem</t>
         </is>
       </c>
     </row>
@@ -12500,10 +12652,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E502" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E502" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="503">
@@ -12529,7 +12680,7 @@
       </c>
       <c r="E503" s="4" t="inlineStr">
         <is>
-          <t>Vlr Item</t>
+          <t>Valor  do  Item</t>
         </is>
       </c>
     </row>
@@ -12556,7 +12707,7 @@
       </c>
       <c r="E504" s="4" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>Código Nacional de Localidade (CNL) (não será impresso)</t>
         </is>
       </c>
     </row>
@@ -12583,7 +12734,7 @@
       </c>
       <c r="E505" s="4" t="inlineStr">
         <is>
-          <t>Nº Contrato</t>
+          <t>Número contrato de vendas</t>
         </is>
       </c>
     </row>
@@ -12610,7 +12761,7 @@
       </c>
       <c r="E506" s="4" t="inlineStr">
         <is>
-          <t>Vlr Imposto</t>
+          <t>Valor do Imposto</t>
         </is>
       </c>
     </row>
@@ -12637,7 +12788,7 @@
       </c>
       <c r="E507" s="4" t="inlineStr">
         <is>
-          <t>Vlr PIS</t>
+          <t>Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -12664,7 +12815,7 @@
       </c>
       <c r="E508" s="4" t="inlineStr">
         <is>
-          <t>Vlr COFINS</t>
+          <t>Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -12691,7 +12842,7 @@
       </c>
       <c r="E509" s="4" t="inlineStr">
         <is>
-          <t>Nº Seq Item</t>
+          <t>Número sequencial do item na nota fiscal/NFCOM.</t>
         </is>
       </c>
     </row>
@@ -12718,7 +12869,7 @@
       </c>
       <c r="E510" s="4" t="inlineStr">
         <is>
-          <t>Cód CFOP</t>
+          <t>Código CFOP. Preencher conforme obrigatoriedade parametrizada na tabela de classificação (cClass).</t>
         </is>
       </c>
     </row>
@@ -12745,7 +12896,7 @@
       </c>
       <c r="E511" s="4" t="inlineStr">
         <is>
-          <t>Unid Medida</t>
+          <t>Unidade Básica de Medida.</t>
         </is>
       </c>
     </row>
@@ -12772,7 +12923,7 @@
       </c>
       <c r="E512" s="4" t="inlineStr">
         <is>
-          <t>Qtd Faturada</t>
+          <t>Quantidade Faturada</t>
         </is>
       </c>
     </row>
@@ -12799,7 +12950,7 @@
       </c>
       <c r="E513" s="4" t="inlineStr">
         <is>
-          <t>Vlr Unit</t>
+          <t>Valor unitário do item</t>
         </is>
       </c>
     </row>
@@ -12826,7 +12977,7 @@
       </c>
       <c r="E514" s="4" t="inlineStr">
         <is>
-          <t>Vlr Desc</t>
+          <t>Valor do Desconto</t>
         </is>
       </c>
     </row>
@@ -12853,7 +13004,7 @@
       </c>
       <c r="E515" s="4" t="inlineStr">
         <is>
-          <t>Base ICMS</t>
+          <t>Valor da Base de Cálculo (Base ICMS)</t>
         </is>
       </c>
     </row>
@@ -12884,12 +13035,17 @@
         </is>
       </c>
     </row>
+    <row r="517"/>
     <row r="518" ht="25" customHeight="1">
       <c r="A518" s="3" t="inlineStr">
         <is>
           <t>REG 48 - Base NFCOM</t>
         </is>
       </c>
+      <c r="B518" s="6" t="n"/>
+      <c r="C518" s="6" t="n"/>
+      <c r="D518" s="6" t="n"/>
+      <c r="E518" s="7" t="n"/>
     </row>
     <row r="519">
       <c r="A519" s="4" t="inlineStr">
@@ -12914,7 +13070,7 @@
       </c>
       <c r="E519" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 48</t>
+          <t>Tipo de Registro = 48</t>
         </is>
       </c>
     </row>
@@ -12939,10 +13095,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E520" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E520" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="521">
@@ -12968,7 +13123,7 @@
       </c>
       <c r="E521" s="4" t="inlineStr">
         <is>
-          <t>Vlr Total</t>
+          <t>Valor  Total</t>
         </is>
       </c>
     </row>
@@ -12993,10 +13148,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E522" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E522" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="523">
@@ -13022,7 +13176,7 @@
       </c>
       <c r="E523" s="4" t="inlineStr">
         <is>
-          <t>Base Cálc</t>
+          <t>Valor da Base de Cálculo</t>
         </is>
       </c>
     </row>
@@ -13049,7 +13203,7 @@
       </c>
       <c r="E524" s="4" t="inlineStr">
         <is>
-          <t>Asterisco</t>
+          <t>Asterisco Alíquota. Preenchido quando existir redução de base de cálculo (**)</t>
         </is>
       </c>
     </row>
@@ -13101,10 +13255,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E526" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E526" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="527">
@@ -13130,7 +13283,7 @@
       </c>
       <c r="E527" s="4" t="inlineStr">
         <is>
-          <t>Vlr ICMS</t>
+          <t>Valor  do  Imposto (ICMS)</t>
         </is>
       </c>
     </row>
@@ -13155,10 +13308,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E528" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E528" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="529">
@@ -13184,7 +13336,7 @@
       </c>
       <c r="E529" s="4" t="inlineStr">
         <is>
-          <t>Vlr Isentos</t>
+          <t>Valor  Isentos</t>
         </is>
       </c>
     </row>
@@ -13209,10 +13361,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E530" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E530" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="531">
@@ -13238,7 +13389,7 @@
       </c>
       <c r="E531" s="4" t="inlineStr">
         <is>
-          <t>Vlr Outros</t>
+          <t>Valor  Outros</t>
         </is>
       </c>
     </row>
@@ -13265,7 +13416,7 @@
       </c>
       <c r="E532" s="4" t="inlineStr">
         <is>
-          <t>Tot Vlr Unit</t>
+          <t>Total Valor unitário</t>
         </is>
       </c>
     </row>
@@ -13292,7 +13443,7 @@
       </c>
       <c r="E533" s="4" t="inlineStr">
         <is>
-          <t>Tot Desc</t>
+          <t>Total Valor do desconto</t>
         </is>
       </c>
     </row>
@@ -13319,7 +13470,7 @@
       </c>
       <c r="E534" s="4" t="inlineStr">
         <is>
-          <t>Tot PIS</t>
+          <t>Total Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -13346,7 +13497,7 @@
       </c>
       <c r="E535" s="4" t="inlineStr">
         <is>
-          <t>Tot COFINS</t>
+          <t>Total Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -13373,7 +13524,7 @@
       </c>
       <c r="E536" s="4" t="inlineStr">
         <is>
-          <t>Tot FUST</t>
+          <t>Total Valor do FUST</t>
         </is>
       </c>
     </row>
@@ -13400,7 +13551,7 @@
       </c>
       <c r="E537" s="4" t="inlineStr">
         <is>
-          <t>Tot FUNTEL</t>
+          <t>Total Valor do FUNTEL</t>
         </is>
       </c>
     </row>
@@ -13431,12 +13582,17 @@
         </is>
       </c>
     </row>
+    <row r="539"/>
     <row r="540" ht="25" customHeight="1">
       <c r="A540" s="3" t="inlineStr">
         <is>
           <t>REG 50 - Somatórios NFCOM</t>
         </is>
       </c>
+      <c r="B540" s="6" t="n"/>
+      <c r="C540" s="6" t="n"/>
+      <c r="D540" s="6" t="n"/>
+      <c r="E540" s="7" t="n"/>
     </row>
     <row r="541">
       <c r="A541" s="4" t="inlineStr">
@@ -13461,7 +13617,7 @@
       </c>
       <c r="E541" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 50</t>
+          <t>Tipo de Registro = 50</t>
         </is>
       </c>
     </row>
@@ -13486,10 +13642,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E542" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E542" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="543">
@@ -13515,7 +13670,7 @@
       </c>
       <c r="E543" s="4" t="inlineStr">
         <is>
-          <t>Som Total</t>
+          <t>Somatório Valor Total</t>
         </is>
       </c>
     </row>
@@ -13540,10 +13695,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E544" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E544" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="545">
@@ -13569,7 +13723,7 @@
       </c>
       <c r="E545" s="4" t="inlineStr">
         <is>
-          <t>Som Base</t>
+          <t>Somatório Valor da Base de Cálculo</t>
         </is>
       </c>
     </row>
@@ -13594,10 +13748,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E546" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E546" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="547">
@@ -13623,7 +13776,7 @@
       </c>
       <c r="E547" s="4" t="inlineStr">
         <is>
-          <t>Som Imposto</t>
+          <t>Somatório Valor de Imposto</t>
         </is>
       </c>
     </row>
@@ -13648,10 +13801,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E548" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E548" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="549">
@@ -13677,7 +13829,7 @@
       </c>
       <c r="E549" s="4" t="inlineStr">
         <is>
-          <t>Som Isentos</t>
+          <t>Somatório Valor Isentos</t>
         </is>
       </c>
     </row>
@@ -13702,10 +13854,9 @@
           <t>X(01)</t>
         </is>
       </c>
-      <c r="E550" s="4" t="inlineStr">
-        <is>
-          <t>C/D</t>
-        </is>
+      <c r="E550" s="4">
+        <f> C, Quando  o  valor for negativo,= D, Quando  o  valor for positivo</f>
+        <v/>
       </c>
     </row>
     <row r="551">
@@ -13731,7 +13882,7 @@
       </c>
       <c r="E551" s="4" t="inlineStr">
         <is>
-          <t>Som Outros</t>
+          <t>Somatório Valor Outros</t>
         </is>
       </c>
     </row>
@@ -13758,7 +13909,7 @@
       </c>
       <c r="E552" s="4" t="inlineStr">
         <is>
-          <t>Hash-Code</t>
+          <t>Hash-Code editado</t>
         </is>
       </c>
     </row>
@@ -13785,7 +13936,7 @@
       </c>
       <c r="E553" s="4" t="inlineStr">
         <is>
-          <t>Tot Unit</t>
+          <t>Total Valor unitário</t>
         </is>
       </c>
     </row>
@@ -13812,7 +13963,7 @@
       </c>
       <c r="E554" s="4" t="inlineStr">
         <is>
-          <t>Tot Desc</t>
+          <t>Total Valor do desconto</t>
         </is>
       </c>
     </row>
@@ -13839,7 +13990,7 @@
       </c>
       <c r="E555" s="4" t="inlineStr">
         <is>
-          <t>Tot PIS</t>
+          <t>Total Valor do PIS</t>
         </is>
       </c>
     </row>
@@ -13866,7 +14017,7 @@
       </c>
       <c r="E556" s="4" t="inlineStr">
         <is>
-          <t>Tot COFINS</t>
+          <t>Total Valor do COFINS</t>
         </is>
       </c>
     </row>
@@ -13893,7 +14044,7 @@
       </c>
       <c r="E557" s="4" t="inlineStr">
         <is>
-          <t>Tot FUST</t>
+          <t>Total Valor do FUST</t>
         </is>
       </c>
     </row>
@@ -13920,7 +14071,7 @@
       </c>
       <c r="E558" s="4" t="inlineStr">
         <is>
-          <t>Tot FUNTEL</t>
+          <t>Total Valor do FUNTEL</t>
         </is>
       </c>
     </row>
@@ -13947,7 +14098,7 @@
       </c>
       <c r="E559" s="4" t="inlineStr">
         <is>
-          <t>Tot PIS Ret</t>
+          <t>Total Valor  do PIS retido</t>
         </is>
       </c>
     </row>
@@ -13974,7 +14125,7 @@
       </c>
       <c r="E560" s="4" t="inlineStr">
         <is>
-          <t>Tot COF Ret</t>
+          <t>Total Valor do COFINS retido</t>
         </is>
       </c>
     </row>
@@ -14001,7 +14152,7 @@
       </c>
       <c r="E561" s="4" t="inlineStr">
         <is>
-          <t>Tot CSLL Ret</t>
+          <t>Total Valor do CSLL retido</t>
         </is>
       </c>
     </row>
@@ -14028,7 +14179,7 @@
       </c>
       <c r="E562" s="4" t="inlineStr">
         <is>
-          <t>Tot IR Ret</t>
+          <t>Total Valor do IR retido</t>
         </is>
       </c>
     </row>
@@ -14059,12 +14210,17 @@
         </is>
       </c>
     </row>
+    <row r="564"/>
     <row r="565" ht="25" customHeight="1">
       <c r="A565" s="3" t="inlineStr">
         <is>
           <t>REG 52 - QRCode PIX</t>
         </is>
       </c>
+      <c r="B565" s="6" t="n"/>
+      <c r="C565" s="6" t="n"/>
+      <c r="D565" s="6" t="n"/>
+      <c r="E565" s="7" t="n"/>
     </row>
     <row r="566">
       <c r="A566" s="4" t="inlineStr">
@@ -14089,7 +14245,7 @@
       </c>
       <c r="E566" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 52</t>
+          <t>Tipo de Registro = 52</t>
         </is>
       </c>
     </row>
@@ -14116,7 +14272,7 @@
       </c>
       <c r="E567" s="4" t="inlineStr">
         <is>
-          <t>URL QRCode PIX (2000b total, 8 regs max)</t>
+          <t>URL do QRCode do PIX apresentado na fatura.</t>
         </is>
       </c>
     </row>
@@ -14143,16 +14299,21 @@
       </c>
       <c r="E568" s="4" t="inlineStr">
         <is>
-          <t>Filler</t>
-        </is>
-      </c>
-    </row>
+          <t>Filler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="569"/>
     <row r="570" ht="25" customHeight="1">
       <c r="A570" s="3" t="inlineStr">
         <is>
           <t>REG 60-68 + 70-82 + 85-88</t>
         </is>
       </c>
+      <c r="B570" s="6" t="n"/>
+      <c r="C570" s="6" t="n"/>
+      <c r="D570" s="6" t="n"/>
+      <c r="E570" s="7" t="n"/>
     </row>
     <row r="571">
       <c r="A571" s="4" t="inlineStr">
@@ -14181,12 +14342,17 @@
         </is>
       </c>
     </row>
+    <row r="572"/>
     <row r="573" ht="25" customHeight="1">
       <c r="A573" s="3" t="inlineStr">
         <is>
           <t>REG 99 - Trailer</t>
         </is>
       </c>
+      <c r="B573" s="6" t="n"/>
+      <c r="C573" s="6" t="n"/>
+      <c r="D573" s="6" t="n"/>
+      <c r="E573" s="7" t="n"/>
     </row>
     <row r="574">
       <c r="A574" s="4" t="inlineStr">
@@ -14211,7 +14377,7 @@
       </c>
       <c r="E574" s="4" t="inlineStr">
         <is>
-          <t>Tipo = 99</t>
+          <t>Tipo de Registro = 99</t>
         </is>
       </c>
     </row>
@@ -14238,7 +14404,7 @@
       </c>
       <c r="E575" s="4" t="inlineStr">
         <is>
-          <t>Total Registros</t>
+          <t>Total de Registros do Arquivo, inclusive com Header  e  Trailler</t>
         </is>
       </c>
     </row>

</xml_diff>